<commit_message>
feat: complete Gradio dashboard with human-guided prompt healing, before/after diff visualizer, and multi-problem test suite
</commit_message>
<xml_diff>
--- a/issues/issues.xlsx
+++ b/issues/issues.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -651,7 +651,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Application form has 'AADHAAR-8921-4321-9988' while ID proof has '8921-4321-9988'. Validator prompt needs generic instruction to normalize common identity prefixes before matching.</t>
+          <t>Application form has 'AADHAAR-8921-4321-9988' while ID proof has '8921-4321-9988'. Validator prompt needs instruction to normalize common identity prefixes before matching.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -676,6 +676,104 @@
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>validate_ticket</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>currency_formatting</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Currency notation discrepancies ('Rs. 3,75,000/-' vs 'INR 375000') flagged as amount mismatch</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Validator treats text formatting difference as conflicting budget amounts instead of recognizing monetary equivalence.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>case_demo_currency_format</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Validator must parse numeric value and recognize that 'Rs. 3,75,000/-' equals 'INR 375000'.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>validate_ticket</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>same_day_dates</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Same-day administrative sanction flagged as suspicious chronological ordering</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Validator strictly expects sanction date strictly before application date without permitting same-day administrative sanction.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>case_demo_date_order</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Validator must allow same-day sanction order and application submission.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add dual Groq API keys support separating Ticket Agent and Testing Agent quotas
</commit_message>
<xml_diff>
--- a/issues/issues.xlsx
+++ b/issues/issues.xlsx
@@ -568,15 +568,19 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>needs_human</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Could not resolve within attempt limit without regressions.</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
fix(ci): fix ModuleNotFoundError for tests_agent in GitHub Actions and add root fix_agent.py
</commit_message>
<xml_diff>
--- a/issues/issues.xlsx
+++ b/issues/issues.xlsx
@@ -568,17 +568,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>needs_human</t>
+          <t>fixing</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Could not resolve within attempt limit without regressions.</t>
+          <t>Proposal error: Failed to obtain prompt fix proposal from Groq.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -719,15 +719,19 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>needs_human</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Could not resolve within attempt limit without regressions.</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
fix(gradio): resolve diff language error and add previous/current prompt viewers
</commit_message>
<xml_diff>
--- a/issues/issues.xlsx
+++ b/issues/issues.xlsx
@@ -568,17 +568,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>fixing</t>
+          <t>fixed</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Proposal error: Failed to obtain prompt fix proposal from Groq.</t>
+          <t>Prompt successfully fixed on attempt 2. Passed issue verification and canonical regression checks.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>

</xml_diff>